<commit_message>
Fix xlsx: fill ER% rows 25-29, move 備註 to last column
</commit_message>
<xml_diff>
--- a/志明AI實驗數據_6_1-6_25.xlsx
+++ b/志明AI實驗數據_6_1-6_25.xlsx
@@ -434,16 +434,16 @@
         <v>分類</v>
       </c>
       <c r="K1" t="str">
+        <v>圖像ER%</v>
+      </c>
+      <c r="L1" t="str">
+        <v>連結ER%</v>
+      </c>
+      <c r="M1" t="str">
+        <v>ER差距(pp)</v>
+      </c>
+      <c r="N1" t="str">
         <v>備註</v>
-      </c>
-      <c r="L1" t="str">
-        <v>圖像ER%</v>
-      </c>
-      <c r="M1" t="str">
-        <v>連結ER%</v>
-      </c>
-      <c r="N1" t="str">
-        <v>ER差距(pp)</v>
       </c>
     </row>
     <row r="2">
@@ -477,17 +477,17 @@
       <c r="J2" t="str">
         <v>財經</v>
       </c>
-      <c r="K2" t="str">
+      <c r="K2">
+        <v>0.551</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0.551</v>
+      </c>
+      <c r="N2" t="str">
         <v>圖像欄為瀏覽人數</v>
-      </c>
-      <c r="L2">
-        <v>0.551</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0.551</v>
       </c>
     </row>
     <row r="3">
@@ -521,17 +521,17 @@
       <c r="J3" t="str">
         <v>財經</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
+      <c r="K3">
+        <v>1.887</v>
       </c>
       <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
         <v>1.887</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>1.887</v>
+      <c r="N3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -565,17 +565,17 @@
       <c r="J4" t="str">
         <v>環境</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
+      <c r="K4">
+        <v>1.515</v>
       </c>
       <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>1.515</v>
       </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>1.515</v>
+      <c r="N4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -609,17 +609,17 @@
       <c r="J5" t="str">
         <v>環境</v>
       </c>
-      <c r="K5" t="str">
-        <v/>
+      <c r="K5">
+        <v>0.64</v>
       </c>
       <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
         <v>0.64</v>
       </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0.64</v>
+      <c r="N5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -653,17 +653,17 @@
       <c r="J6" t="str">
         <v>政治</v>
       </c>
-      <c r="K6" t="str">
-        <v/>
+      <c r="K6">
+        <v>0.948</v>
       </c>
       <c r="L6">
-        <v>0.948</v>
+        <v>0.377</v>
       </c>
       <c r="M6">
-        <v>0.377</v>
-      </c>
-      <c r="N6">
         <v>0.571</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -697,17 +697,17 @@
       <c r="J7" t="str">
         <v>政治</v>
       </c>
-      <c r="K7" t="str">
-        <v/>
+      <c r="K7">
+        <v>27.273</v>
       </c>
       <c r="L7">
-        <v>27.273</v>
+        <v>20</v>
       </c>
       <c r="M7">
-        <v>20</v>
-      </c>
-      <c r="N7">
         <v>7.273</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -741,17 +741,17 @@
       <c r="J8" t="str">
         <v>政治</v>
       </c>
-      <c r="K8" t="str">
-        <v/>
+      <c r="K8">
+        <v>0.851</v>
       </c>
       <c r="L8">
-        <v>0.851</v>
+        <v>0.909</v>
       </c>
       <c r="M8">
-        <v>0.909</v>
-      </c>
-      <c r="N8">
         <v>-0.058</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -785,17 +785,17 @@
       <c r="J9" t="str">
         <v>政治</v>
       </c>
-      <c r="K9" t="str">
-        <v/>
+      <c r="K9">
+        <v>2.137</v>
       </c>
       <c r="L9">
-        <v>2.137</v>
+        <v>0.943</v>
       </c>
       <c r="M9">
-        <v>0.943</v>
-      </c>
-      <c r="N9">
         <v>1.194</v>
+      </c>
+      <c r="N9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -829,17 +829,17 @@
       <c r="J10" t="str">
         <v>社會</v>
       </c>
-      <c r="K10" t="str">
-        <v/>
+      <c r="K10">
+        <v>2.343</v>
       </c>
       <c r="L10">
-        <v>2.343</v>
+        <v>2.381</v>
       </c>
       <c r="M10">
-        <v>2.381</v>
-      </c>
-      <c r="N10">
         <v>-0.038</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -873,17 +873,17 @@
       <c r="J11" t="str">
         <v>社會</v>
       </c>
-      <c r="K11" t="str">
+      <c r="K11">
+        <v>0.314</v>
+      </c>
+      <c r="L11">
+        <v>0.732</v>
+      </c>
+      <c r="M11">
+        <v>-0.418</v>
+      </c>
+      <c r="N11" t="str">
         <v>互動差距 1，同豬肉情況</v>
-      </c>
-      <c r="L11">
-        <v>0.314</v>
-      </c>
-      <c r="M11">
-        <v>0.732</v>
-      </c>
-      <c r="N11">
-        <v>-0.418</v>
       </c>
     </row>
     <row r="12">
@@ -917,17 +917,17 @@
       <c r="J12" t="str">
         <v>社會</v>
       </c>
-      <c r="K12" t="str">
-        <v/>
+      <c r="K12">
+        <v>1.406</v>
       </c>
       <c r="L12">
-        <v>1.406</v>
+        <v>1.235</v>
       </c>
       <c r="M12">
-        <v>1.235</v>
-      </c>
-      <c r="N12">
         <v>0.171</v>
+      </c>
+      <c r="N12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -961,17 +961,17 @@
       <c r="J13" t="str">
         <v>社會</v>
       </c>
-      <c r="K13" t="str">
-        <v/>
+      <c r="K13">
+        <v>1.083</v>
       </c>
       <c r="L13">
-        <v>1.083</v>
+        <v>1.205</v>
       </c>
       <c r="M13">
-        <v>1.205</v>
-      </c>
-      <c r="N13">
         <v>-0.122</v>
+      </c>
+      <c r="N13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1005,17 +1005,17 @@
       <c r="J14" t="str">
         <v>政治</v>
       </c>
-      <c r="K14" t="str">
-        <v/>
+      <c r="K14">
+        <v>0.987</v>
       </c>
       <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
         <v>0.987</v>
       </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0.987</v>
+      <c r="N14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1049,17 +1049,17 @@
       <c r="J15" t="str">
         <v>環境</v>
       </c>
-      <c r="K15" t="str">
-        <v/>
+      <c r="K15">
+        <v>0.826</v>
       </c>
       <c r="L15">
-        <v>0.826</v>
+        <v>0.87</v>
       </c>
       <c r="M15">
-        <v>0.87</v>
-      </c>
-      <c r="N15">
         <v>-0.044</v>
+      </c>
+      <c r="N15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1093,17 +1093,17 @@
       <c r="J16" t="str">
         <v>財經</v>
       </c>
-      <c r="K16" t="str">
+      <c r="K16">
+        <v>0.475</v>
+      </c>
+      <c r="L16">
+        <v>1.158</v>
+      </c>
+      <c r="M16">
+        <v>-0.683</v>
+      </c>
+      <c r="N16" t="str">
         <v>互動差距 1，視為持平</v>
-      </c>
-      <c r="L16">
-        <v>0.475</v>
-      </c>
-      <c r="M16">
-        <v>1.158</v>
-      </c>
-      <c r="N16">
-        <v>-0.683</v>
       </c>
     </row>
     <row r="17">
@@ -1137,17 +1137,17 @@
       <c r="J17" t="str">
         <v>社會</v>
       </c>
-      <c r="K17" t="str">
-        <v/>
+      <c r="K17">
+        <v>1.195</v>
       </c>
       <c r="L17">
-        <v>1.195</v>
+        <v>1.604</v>
       </c>
       <c r="M17">
-        <v>1.604</v>
-      </c>
-      <c r="N17">
         <v>-0.409</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1181,17 +1181,17 @@
       <c r="J18" t="str">
         <v>社會</v>
       </c>
-      <c r="K18" t="str">
-        <v/>
+      <c r="K18">
+        <v>16.667</v>
       </c>
       <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
         <v>16.667</v>
       </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>16.667</v>
+      <c r="N18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1225,17 +1225,17 @@
       <c r="J19" t="str">
         <v>政治</v>
       </c>
-      <c r="K19" t="str">
-        <v/>
+      <c r="K19">
+        <v>1.232</v>
       </c>
       <c r="L19">
-        <v>1.232</v>
+        <v>1.176</v>
       </c>
       <c r="M19">
-        <v>1.176</v>
-      </c>
-      <c r="N19">
         <v>0.056</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1269,17 +1269,17 @@
       <c r="J20" t="str">
         <v>社會</v>
       </c>
-      <c r="K20" t="str">
-        <v/>
+      <c r="K20">
+        <v>0.714</v>
       </c>
       <c r="L20">
-        <v>0.714</v>
+        <v>1.389</v>
       </c>
       <c r="M20">
-        <v>1.389</v>
-      </c>
-      <c r="N20">
         <v>-0.675</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1313,17 +1313,17 @@
       <c r="J21" t="str">
         <v>文化</v>
       </c>
-      <c r="K21" t="str">
-        <v/>
+      <c r="K21">
+        <v>0.588</v>
       </c>
       <c r="L21">
-        <v>0.588</v>
+        <v>1.282</v>
       </c>
       <c r="M21">
-        <v>1.282</v>
-      </c>
-      <c r="N21">
         <v>-0.694</v>
+      </c>
+      <c r="N21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1357,17 +1357,17 @@
       <c r="J22" t="str">
         <v>財經</v>
       </c>
-      <c r="K22" t="str">
-        <v/>
+      <c r="K22">
+        <v>1.282</v>
       </c>
       <c r="L22">
-        <v>1.282</v>
+        <v>2.256</v>
       </c>
       <c r="M22">
-        <v>2.256</v>
-      </c>
-      <c r="N22">
         <v>-0.974</v>
+      </c>
+      <c r="N22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1401,17 +1401,17 @@
       <c r="J23" t="str">
         <v>社會</v>
       </c>
-      <c r="K23" t="str">
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0.69</v>
+      </c>
+      <c r="M23">
+        <v>-0.69</v>
+      </c>
+      <c r="N23" t="str">
         <v>首次連結勝</v>
-      </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
-        <v>0.69</v>
-      </c>
-      <c r="N23">
-        <v>-0.69</v>
       </c>
     </row>
     <row r="24">
@@ -1445,17 +1445,17 @@
       <c r="J24" t="str">
         <v>科技</v>
       </c>
-      <c r="K24" t="str">
-        <v/>
+      <c r="K24">
+        <v>1.227</v>
       </c>
       <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
         <v>1.227</v>
       </c>
-      <c r="M24">
-        <v>0</v>
-      </c>
-      <c r="N24">
-        <v>1.227</v>
+      <c r="N24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1489,17 +1489,17 @@
       <c r="J25" t="str">
         <v>環境</v>
       </c>
-      <c r="K25" t="str">
-        <v/>
+      <c r="K25">
+        <v>0.829</v>
       </c>
       <c r="L25">
-        <v>0.829</v>
+        <v>1.099</v>
       </c>
       <c r="M25">
-        <v>1.099</v>
-      </c>
-      <c r="N25">
         <v>-0.27</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1533,14 +1533,14 @@
       <c r="J26" t="str">
         <v>社會</v>
       </c>
-      <c r="K26" t="str">
-        <v/>
-      </c>
-      <c r="L26" t="str">
-        <v/>
-      </c>
-      <c r="M26" t="str">
-        <v/>
+      <c r="K26">
+        <v>1.401</v>
+      </c>
+      <c r="L26">
+        <v>1.763</v>
+      </c>
+      <c r="M26">
+        <v>-0.362</v>
       </c>
       <c r="N26" t="str">
         <v/>
@@ -1577,17 +1577,17 @@
       <c r="J27" t="str">
         <v>財經</v>
       </c>
-      <c r="K27" t="str">
+      <c r="K27">
+        <v>0.439</v>
+      </c>
+      <c r="L27">
+        <v>0.546</v>
+      </c>
+      <c r="M27">
+        <v>-0.107</v>
+      </c>
+      <c r="N27" t="str">
         <v>4變體取最佳圖像(D)vs連結(B)，持平</v>
-      </c>
-      <c r="L27" t="str">
-        <v/>
-      </c>
-      <c r="M27" t="str">
-        <v/>
-      </c>
-      <c r="N27" t="str">
-        <v/>
       </c>
     </row>
     <row r="28">
@@ -1621,17 +1621,17 @@
       <c r="J28" t="str">
         <v>政治</v>
       </c>
-      <c r="K28" t="str">
+      <c r="K28">
+        <v>1.484</v>
+      </c>
+      <c r="L28">
+        <v>0.806</v>
+      </c>
+      <c r="M28">
+        <v>0.678</v>
+      </c>
+      <c r="N28" t="str">
         <v>最佳圖像 vs 連結</v>
-      </c>
-      <c r="L28" t="str">
-        <v/>
-      </c>
-      <c r="M28" t="str">
-        <v/>
-      </c>
-      <c r="N28" t="str">
-        <v/>
       </c>
     </row>
     <row r="29">
@@ -1665,14 +1665,14 @@
       <c r="J29" t="str">
         <v>社會</v>
       </c>
-      <c r="K29" t="str">
-        <v/>
-      </c>
-      <c r="L29" t="str">
-        <v/>
-      </c>
-      <c r="M29" t="str">
-        <v/>
+      <c r="K29">
+        <v>1.116</v>
+      </c>
+      <c r="L29">
+        <v>1.887</v>
+      </c>
+      <c r="M29">
+        <v>-0.771</v>
       </c>
       <c r="N29" t="str">
         <v/>
@@ -1709,17 +1709,17 @@
       <c r="J30" t="str">
         <v>社會</v>
       </c>
-      <c r="K30" t="str">
+      <c r="K30">
+        <v>4.172</v>
+      </c>
+      <c r="L30">
+        <v>1.205</v>
+      </c>
+      <c r="M30">
+        <v>2.967</v>
+      </c>
+      <c r="N30" t="str">
         <v>4變體取最佳圖像(A)vs連結(B)</v>
-      </c>
-      <c r="L30" t="str">
-        <v/>
-      </c>
-      <c r="M30" t="str">
-        <v/>
-      </c>
-      <c r="N30" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>